<commit_message>
Preserve P-1 row identity
</commit_message>
<xml_diff>
--- a/dod_ic_budget_analyzer/tests/fixtures/p1_fy2027_sample.xlsx
+++ b/dod_ic_budget_analyzer/tests/fixtures/p1_fy2027_sample.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exhibit P-1" sheetId="1" r:id="R4d2e18f6f79042d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exhibit P-1" sheetId="1" r:id="Rd57d62c276e340b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -997,6 +997,142 @@
         <x:v>U</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" ht="18" customHeight="1">
+      <x:c r="A9" t="str">
+        <x:v>2031A</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Aircraft Procurement, Army</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Aircraft</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Fixed Wing</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>9670A00005</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>MQ-1 UAV</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>Less: Advance Procurement (PY)</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>Add</x:v>
+      </x:c>
+      <x:c r="N9"/>
+      <x:c r="O9"/>
+      <x:c r="P9"/>
+      <x:c r="Q9"/>
+      <x:c r="R9"/>
+      <x:c r="S9"/>
+      <x:c r="T9"/>
+      <x:c r="U9" t="n">
+        <x:v>-40000</x:v>
+      </x:c>
+      <x:c r="V9"/>
+      <x:c r="W9"/>
+      <x:c r="X9"/>
+      <x:c r="Y9" t="n">
+        <x:v>-40000</x:v>
+      </x:c>
+      <x:c r="Z9"/>
+      <x:c r="AA9"/>
+      <x:c r="AB9"/>
+      <x:c r="AC9"/>
+      <x:c r="AD9"/>
+      <x:c r="AE9"/>
+      <x:c r="AF9" t="str">
+        <x:v>U</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="18" customHeight="1">
+      <x:c r="A10" t="str">
+        <x:v>2031A</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Aircraft Procurement, Army</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>05</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Modification of inservice aircraft</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Tactical Aircraft</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>9670A00005</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>MQ-1 UAV</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>Weapon System Cost</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>Add</x:v>
+      </x:c>
+      <x:c r="N10"/>
+      <x:c r="O10"/>
+      <x:c r="P10"/>
+      <x:c r="Q10"/>
+      <x:c r="R10"/>
+      <x:c r="S10"/>
+      <x:c r="T10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U10" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="V10"/>
+      <x:c r="W10"/>
+      <x:c r="X10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y10" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="Z10"/>
+      <x:c r="AA10"/>
+      <x:c r="AB10"/>
+      <x:c r="AC10"/>
+      <x:c r="AD10"/>
+      <x:c r="AE10"/>
+      <x:c r="AF10" t="str">
+        <x:v>U</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>